<commit_message>
feat(productos): Kit de Tareas Catering — el 09 pasa de caja de mostrador a «Cobros y Facturación por Evento» (antes/después del evento, liquidación con IVA 10/21, anticipo, pendiente y estado VENCIDO, registro de 25 eventos; barra en efectivo opcional) con redirect del fichero antiguo; 347 tareas. Metadata subject/title v2.0 en los 55 xlsx P4 de hotel, chocolatería, heladería y restaurante-creativo (motor 2.5); hotel sin el «46 checklists» en título, subject y dashboard (son 53 en 19 ficheros). Censo 0, gate offline 44/647/0
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/astro-site/public/dl/kit-tareas-catering/03-tareas-manager.xlsx
+++ b/astro-site/public/dl/kit-tareas-catering/03-tareas-manager.xlsx
@@ -1589,9 +1589,9 @@
   </sheetData>
   <mergeCells count="8">
     <mergeCell ref="A4:G4"/>
+    <mergeCell ref="A15:G15"/>
+    <mergeCell ref="A1:G1"/>
     <mergeCell ref="A49:G49"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A15:G15"/>
     <mergeCell ref="A50:G50"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A27:G27"/>
@@ -1627,7 +1627,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G50"/>
+  <dimension ref="A1:G37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2327,26 +2327,13 @@
         </is>
       </c>
     </row>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
   </sheetData>
   <mergeCells count="8">
     <mergeCell ref="A4:G4"/>
     <mergeCell ref="A28:G28"/>
+    <mergeCell ref="A1:G1"/>
     <mergeCell ref="A36:G36"/>
     <mergeCell ref="A37:G37"/>
-    <mergeCell ref="A1:G1"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A21:G21"/>
     <mergeCell ref="A13:G13"/>

</xml_diff>